<commit_message>
Sync Gantt and research canvas with notes, slides, and notebook
Gantt: mark pilot analysis done, map fusion tasks to Stages 2-4, refresh
follow-up and meeting wording, point Notes sheet at Stage1_refactor.
Canvas: Stage 1 pilot results header, Stages 2-4 methods line, Coupled
Mamba described as needing no alignment loss. Notes and slide 3 aligned
on the same Coupled Mamba wording; slide 3 codon-grid and Q2 tags fixed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PDtcWBhFCqkHgy4GaB1JdB
</commit_message>
<xml_diff>
--- a/Notes/Research_Project_Plan_Gantt_McKinley.xlsx
+++ b/Notes/Research_Project_Plan_Gantt_McKinley.xlsx
@@ -101,7 +101,7 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">Progress meeting with Mina (1-2 slides)</t>
+    <t xml:space="preserve">Progress meeting with Mina (Stage 1 results)</t>
   </si>
   <si>
     <t xml:space="preserve">Planned</t>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Scale Stage 1 to full ~41K mRNA Stability set and mRFP Expression labels</t>
   </si>
   <si>
-    <t xml:space="preserve">Interpretability follow-ups (attention vs. motifs, species subgroup check)</t>
+    <t xml:space="preserve">Interpretability follow-ups (species subgroup check, other attention layers and heads)</t>
   </si>
   <si>
     <t xml:space="preserve">8</t>
@@ -125,34 +125,34 @@
     <t xml:space="preserve">8, 9</t>
   </si>
   <si>
-    <t xml:space="preserve">Stage 2: Fusion and Benchmarking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Codon-level alignment module (resample RNA and protein embeddings)</t>
+    <t xml:space="preserve">Stages 2 to 4: Alignment, Fusion, and Benchmarking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stage 2: codon-grid alignment (resample RNA onto the protein codon grid)</t>
   </si>
   <si>
     <t xml:space="preserve">10</t>
   </si>
   <si>
-    <t xml:space="preserve">Baselines: single-modality and concatenation models</t>
+    <t xml:space="preserve">Stage 3: baselines (single-modality, concatenation + MLP)</t>
   </si>
   <si>
     <t xml:space="preserve">11</t>
   </si>
   <si>
-    <t xml:space="preserve">Cross-attention fusion model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coupled Mamba fusion model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alignment-loss ablation (with vs. without explicit alignment)</t>
+    <t xml:space="preserve">Stage 3: cross-attention fusion model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stage 3: Coupled Mamba fusion model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stage 3: alignment-loss ablation (with vs. without explicit alignment)</t>
   </si>
   <si>
     <t xml:space="preserve">13, 14</t>
   </si>
   <si>
-    <t xml:space="preserve">Benchmark and statistics (5-fold CV, R-squared, Spearman)</t>
+    <t xml:space="preserve">Stage 4: benchmark and statistics (5-fold CV, R-squared, Spearman)</t>
   </si>
   <si>
     <t xml:space="preserve">12, 13, 14, 15</t>
@@ -221,7 +221,7 @@
     <t xml:space="preserve">Work continues after the capstone toward publication (Julian); 2027 dates are targets to confirm with Mina.</t>
   </si>
   <si>
-    <t xml:space="preserve">Stage 1 status reflects Code/Stage1.ipynb as of Sep 22, 2026 (1,000-sequence pilot complete).</t>
+    <t xml:space="preserve">Stage 1 status reflects Code/Stage1_refactor.ipynb as of Sep 23, 2026 (1,000-sequence pilot complete).</t>
   </si>
   <si>
     <t xml:space="preserve">Agentic AI component: required by the capstone course; scope and dates to confirm with the course professor.</t>
@@ -1479,7 +1479,7 @@
         <v>24</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>46279</v>

</xml_diff>